<commit_message>
Add 49 negative test cases to Arteri (rebalance 50/40/10)
</commit_message>
<xml_diff>
--- a/projects/arteri-elearning/test-cases.xlsx
+++ b/projects/arteri-elearning/test-cases.xlsx
@@ -513,7 +513,6 @@
           <t>Document Info</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -609,7 +608,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>70</v>
+        <v>97</v>
       </c>
     </row>
     <row r="13">
@@ -619,7 +618,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>65</v>
+        <v>87</v>
       </c>
     </row>
     <row r="14">
@@ -632,6 +631,7 @@
         <v>135</v>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="18">
@@ -661,7 +661,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
     </row>
     <row r="19">
@@ -671,7 +671,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>27</v>
+        <v>37</v>
       </c>
     </row>
     <row r="20">
@@ -691,9 +691,10 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>14</v>
-      </c>
-    </row>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
@@ -713,7 +714,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>51</v>
+        <v>62</v>
       </c>
     </row>
     <row r="25">
@@ -723,7 +724,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>15</v>
+        <v>29</v>
       </c>
     </row>
     <row r="26">
@@ -733,9 +734,10 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>4</v>
-      </c>
-    </row>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
@@ -829,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L71"/>
+  <dimension ref="A1:L98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4736,6 +4738,1488 @@
       <c r="K71" s="4" t="inlineStr"/>
       <c r="L71" s="4" t="inlineStr"/>
     </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>AUTH-011</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t>Login dengan email mengandung SQL injection</t>
+        </is>
+      </c>
+      <c r="F72" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G72" s="4" t="inlineStr">
+        <is>
+          <t>1. Buka /login
+2. Isi email: ' OR 1=1--
+3. Isi password apa saja
+4. Klik Masuk</t>
+        </is>
+      </c>
+      <c r="H72" s="4" t="inlineStr">
+        <is>
+          <t>Login ditolak, error 'Format email tidak valid' (input disanitasi)</t>
+        </is>
+      </c>
+      <c r="I72" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J72" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K72" s="4" t="inlineStr"/>
+      <c r="L72" s="4" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>AUTH-012</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>Login dengan password mengandung XSS script</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G73" s="4" t="inlineStr">
+        <is>
+          <t>1. Buka /login
+2. Isi email valid
+3. Isi password: &lt;script&gt;alert(1)&lt;/script&gt;
+4. Klik Masuk</t>
+        </is>
+      </c>
+      <c r="H73" s="4" t="inlineStr">
+        <is>
+          <t>Login gagal (kredensial salah), input di-escape, no script execution</t>
+        </is>
+      </c>
+      <c r="I73" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J73" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K73" s="4" t="inlineStr"/>
+      <c r="L73" s="4" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>AUTH-013</t>
+        </is>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>Login</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="inlineStr">
+        <is>
+          <t>Login dengan email lebih dari 255 karakter</t>
+        </is>
+      </c>
+      <c r="F74" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G74" s="4" t="inlineStr">
+        <is>
+          <t>1. Isi email 300 karakter (long string)
+2. Submit</t>
+        </is>
+      </c>
+      <c r="H74" s="4" t="inlineStr">
+        <is>
+          <t>Validasi max length, error 'Email maksimal 255 karakter'</t>
+        </is>
+      </c>
+      <c r="I74" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J74" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K74" s="4" t="inlineStr"/>
+      <c r="L74" s="4" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>AUTH-014</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>JWT dengan signature dimodifikasi (tampered)</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
+          <t>User login</t>
+        </is>
+      </c>
+      <c r="G75" s="4" t="inlineStr">
+        <is>
+          <t>1. Login
+2. Modify signature di localStorage JWT
+3. Refresh page</t>
+        </is>
+      </c>
+      <c r="H75" s="4" t="inlineStr">
+        <is>
+          <t>401 Unauthorized, redirect ke /login (server reject signature)</t>
+        </is>
+      </c>
+      <c r="I75" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J75" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K75" s="4" t="inlineStr"/>
+      <c r="L75" s="4" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t>AUTH-015</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>JWT</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>JWT dengan alg 'none' (algorithm confusion attack)</t>
+        </is>
+      </c>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G76" s="4" t="inlineStr">
+        <is>
+          <t>1. Set localStorage JWT dengan header alg=none
+2. Buka protected route</t>
+        </is>
+      </c>
+      <c r="H76" s="4" t="inlineStr">
+        <is>
+          <t>401 Unauthorized, server reject unsigned token</t>
+        </is>
+      </c>
+      <c r="I76" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J76" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K76" s="4" t="inlineStr"/>
+      <c r="L76" s="4" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>AUTH-016</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>Brute Force</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>Login gagal 10x berturut-turut (brute force)</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G77" s="4" t="inlineStr">
+        <is>
+          <t>1. Buka /login
+2. Submit password salah 10x dalam 5 menit</t>
+        </is>
+      </c>
+      <c r="H77" s="4" t="inlineStr">
+        <is>
+          <t>Setelah 5x: rate limit aktif, response 429 Too Many Requests</t>
+        </is>
+      </c>
+      <c r="I77" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J77" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K77" s="4" t="inlineStr"/>
+      <c r="L77" s="4" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>AUTH-017</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>Cookie</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>Cookie access_token dimanipulasi / dihapus</t>
+        </is>
+      </c>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>User login</t>
+        </is>
+      </c>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
+          <t>1. Login
+2. Hapus cookie access_token via DevTools
+3. Refresh</t>
+        </is>
+      </c>
+      <c r="H78" s="4" t="inlineStr">
+        <is>
+          <t>Middleware tidak bisa decode, redirect ke /login</t>
+        </is>
+      </c>
+      <c r="I78" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J78" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K78" s="4" t="inlineStr"/>
+      <c r="L78" s="4" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>CBT-028</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>CBT</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>Timer</t>
+        </is>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>Timer mundur ke nilai negatif</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>1. Manipulasi timer state ke -1 (via DevTools)</t>
+        </is>
+      </c>
+      <c r="H79" s="4" t="inlineStr">
+        <is>
+          <t>Timer auto-submit, atau UI block invalid state</t>
+        </is>
+      </c>
+      <c r="I79" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J79" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K79" s="4" t="inlineStr"/>
+      <c r="L79" s="4" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>CBT-029</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>CBT</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>Timer</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>Timer window blur (pindah window)，会不会 pause timer</t>
+        </is>
+      </c>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>Exam in progress</t>
+        </is>
+      </c>
+      <c r="G80" s="4" t="inlineStr">
+        <is>
+          <t>1. Pindah window ke aplikasi lain (Alt+Tab)
+2. Tunggu 5 menit
+3. Kembali</t>
+        </is>
+      </c>
+      <c r="H80" s="4" t="inlineStr">
+        <is>
+          <t>Timer TETAP jalan (server-side validation), tidak di-pause oleh blur</t>
+        </is>
+      </c>
+      <c r="I80" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J80" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K80" s="4" t="inlineStr"/>
+      <c r="L80" s="4" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>CBT-030</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>CBT</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>Tab Switch</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>Tab switch &gt; 3x (multiple violations)</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>Sudah 2 lives hilang</t>
+        </is>
+      </c>
+      <c r="G81" s="4" t="inlineStr">
+        <is>
+          <t>1. Switch tab 5x berturut-turut cepat</t>
+        </is>
+      </c>
+      <c r="H81" s="4" t="inlineStr">
+        <is>
+          <t>Semua switch ke-record, lives jadi 0, auto-disqualify</t>
+        </is>
+      </c>
+      <c r="I81" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J81" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K81" s="4" t="inlineStr"/>
+      <c r="L81" s="4" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t>CBT-031</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>CBT</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>Tab Switch</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="inlineStr">
+        <is>
+          <t>Tab switch dengan DevTools disable event listener</t>
+        </is>
+      </c>
+      <c r="F82" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G82" s="4" t="inlineStr">
+        <is>
+          <t>1. Buka DevTools, remove window.blur listener
+2. Switch tab</t>
+        </is>
+      </c>
+      <c r="H82" s="4" t="inlineStr">
+        <is>
+          <t>Backend tetap catat tab switch (server-side validation), lives decrement</t>
+        </is>
+      </c>
+      <c r="I82" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J82" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K82" s="4" t="inlineStr"/>
+      <c r="L82" s="4" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>CBT-032</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>CBT</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>Auto Save</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>Auto-save dengan payload super besar (DoS attempt)</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G83" s="4" t="inlineStr">
+        <is>
+          <t>1. Inject localStorage dengan 100MB data
+2. Trigger auto-save</t>
+        </is>
+      </c>
+      <c r="H83" s="4" t="inlineStr">
+        <is>
+          <t>Auto-save gagal, tidak crash app, error logged, retry dengan snapshot kecil</t>
+        </is>
+      </c>
+      <c r="I83" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J83" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K83" s="4" t="inlineStr"/>
+      <c r="L83" s="4" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>CBT-033</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>CBT</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>Answer State</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="inlineStr">
+        <is>
+          <t>Manipulasi Redux state via DevTools (cheating)</t>
+        </is>
+      </c>
+      <c r="F84" s="4" t="inlineStr">
+        <is>
+          <t>Exam in progress</t>
+        </is>
+      </c>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
+          <t>1. Buka DevTools
+2. Inject jawaban langsung ke Redux state
+3. Submit</t>
+        </is>
+      </c>
+      <c r="H84" s="4" t="inlineStr">
+        <is>
+          <t>Backend verifikasi jawaban dengan attempt_id, hanya jawaban tersimpan yang dihitung</t>
+        </is>
+      </c>
+      <c r="I84" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J84" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K84" s="4" t="inlineStr"/>
+      <c r="L84" s="4" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>CBT-034</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>CBT</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>Resume</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="inlineStr">
+        <is>
+          <t>Resume attempt yang sudah disubmit (race condition)</t>
+        </is>
+      </c>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>1. Submit exam di tab A
+2. Buka tab B, refresh (attempt_id sama)</t>
+        </is>
+      </c>
+      <c r="H85" s="4" t="inlineStr">
+        <is>
+          <t>Tab B: exam sudah disubmit, redirect ke result page</t>
+        </is>
+      </c>
+      <c r="I85" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J85" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K85" s="4" t="inlineStr"/>
+      <c r="L85" s="4" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>CBT-035</t>
+        </is>
+      </c>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>CBT</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>Question</t>
+        </is>
+      </c>
+      <c r="E86" s="4" t="inlineStr">
+        <is>
+          <t>Soal dengan question_type tidak dikenal dari backend</t>
+        </is>
+      </c>
+      <c r="F86" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G86" s="4" t="inlineStr">
+        <is>
+          <t>1. Backend return soal dengan question_type='unknown_type'</t>
+        </is>
+      </c>
+      <c r="H86" s="4" t="inlineStr">
+        <is>
+          <t>Component fallback ke error state, exam tidak crash, soal diskip atau di-flag</t>
+        </is>
+      </c>
+      <c r="I86" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J86" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K86" s="4" t="inlineStr"/>
+      <c r="L86" s="4" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>CBT-036</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>CBT</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>Question</t>
+        </is>
+      </c>
+      <c r="E87" s="4" t="inlineStr">
+        <is>
+          <t>Soal dengan options kosong (corrupt data)</t>
+        </is>
+      </c>
+      <c r="F87" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G87" s="4" t="inlineStr">
+        <is>
+          <t>1. Backend return soal single_choice tanpa options</t>
+        </is>
+      </c>
+      <c r="H87" s="4" t="inlineStr">
+        <is>
+          <t>Soal tampil dengan pesan 'Soal tidak valid', tidak bisa dijawab, flag otomatis</t>
+        </is>
+      </c>
+      <c r="I87" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J87" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K87" s="4" t="inlineStr"/>
+      <c r="L87" s="4" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="inlineStr">
+        <is>
+          <t>CBT-037</t>
+        </is>
+      </c>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>CBT</t>
+        </is>
+      </c>
+      <c r="C88" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>Matching</t>
+        </is>
+      </c>
+      <c r="E88" s="4" t="inlineStr">
+        <is>
+          <t>Soal matching dengan pair tidak lengkap (hanya left atau right)</t>
+        </is>
+      </c>
+      <c r="F88" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G88" s="4" t="inlineStr">
+        <is>
+          <t>1. Backend return soal matching dengan options side=left saja</t>
+        </is>
+      </c>
+      <c r="H88" s="4" t="inlineStr">
+        <is>
+          <t>Service normalize &amp; fallback, soal tetap renderable</t>
+        </is>
+      </c>
+      <c r="I88" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J88" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K88" s="4" t="inlineStr"/>
+      <c r="L88" s="4" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>STU-015</t>
+        </is>
+      </c>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>Student</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>Enroll</t>
+        </is>
+      </c>
+      <c r="E89" s="4" t="inlineStr">
+        <is>
+          <t>Enroll ke course yang tidak ada</t>
+        </is>
+      </c>
+      <c r="F89" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G89" s="4" t="inlineStr">
+        <is>
+          <t>1. POST /student/enroll dengan course_id=99999 (invalid)</t>
+        </is>
+      </c>
+      <c r="H89" s="4" t="inlineStr">
+        <is>
+          <t>404 Not Found, error message 'Course tidak ditemukan'</t>
+        </is>
+      </c>
+      <c r="I89" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J89" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K89" s="4" t="inlineStr"/>
+      <c r="L89" s="4" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="inlineStr">
+        <is>
+          <t>STU-016</t>
+        </is>
+      </c>
+      <c r="B90" s="4" t="inlineStr">
+        <is>
+          <t>Student</t>
+        </is>
+      </c>
+      <c r="C90" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>Enroll</t>
+        </is>
+      </c>
+      <c r="E90" s="4" t="inlineStr">
+        <is>
+          <t>Double enroll (submit form 2x cepat)</t>
+        </is>
+      </c>
+      <c r="F90" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G90" s="4" t="inlineStr">
+        <is>
+          <t>1. Klik Enroll 2x cepat (double-click)</t>
+        </is>
+      </c>
+      <c r="H90" s="4" t="inlineStr">
+        <is>
+          <t>Hanya 1 enroll yang terbuat, idempotent</t>
+        </is>
+      </c>
+      <c r="I90" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J90" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K90" s="4" t="inlineStr"/>
+      <c r="L90" s="4" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <t>STU-017</t>
+        </is>
+      </c>
+      <c r="B91" s="4" t="inlineStr">
+        <is>
+          <t>Student</t>
+        </is>
+      </c>
+      <c r="C91" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>Quiz</t>
+        </is>
+      </c>
+      <c r="E91" s="4" t="inlineStr">
+        <is>
+          <t>Submit quiz tanpa jawab semua soal</t>
+        </is>
+      </c>
+      <c r="F91" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G91" s="4" t="inlineStr">
+        <is>
+          <t>1. Mulai quiz
+2. Submit tanpa jawab semua</t>
+        </is>
+      </c>
+      <c r="H91" s="4" t="inlineStr">
+        <is>
+          <t>Submit tetap sukses, soal unanswered = 0 (atau warning)</t>
+        </is>
+      </c>
+      <c r="I91" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J91" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K91" s="4" t="inlineStr"/>
+      <c r="L91" s="4" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="inlineStr">
+        <is>
+          <t>STU-018</t>
+        </is>
+      </c>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t>Student</t>
+        </is>
+      </c>
+      <c r="C92" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>Quiz</t>
+        </is>
+      </c>
+      <c r="E92" s="4" t="inlineStr">
+        <is>
+          <t>Start quiz yang sudah pernah di-attempt (resume vs new)</t>
+        </is>
+      </c>
+      <c r="F92" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G92" s="4" t="inlineStr">
+        <is>
+          <t>1. Quiz pernah di-start, attempt_id tersimpan
+2. Klik Mulai Quiz lagi</t>
+        </is>
+      </c>
+      <c r="H92" s="4" t="inlineStr">
+        <is>
+          <t>Backend return attempt yang sama (resume), tidak duplicate</t>
+        </is>
+      </c>
+      <c r="I92" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J92" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K92" s="4" t="inlineStr"/>
+      <c r="L92" s="4" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr">
+        <is>
+          <t>STU-019</t>
+        </is>
+      </c>
+      <c r="B93" s="4" t="inlineStr">
+        <is>
+          <t>Student</t>
+        </is>
+      </c>
+      <c r="C93" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>Notifications</t>
+        </is>
+      </c>
+      <c r="E93" s="4" t="inlineStr">
+        <is>
+          <t>Mark as read notifikasi yang sudah dihapus (race)</t>
+        </is>
+      </c>
+      <c r="F93" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G93" s="4" t="inlineStr">
+        <is>
+          <t>1. Hapus notifikasi X
+2. Klik notifikasi X dari cache (sebelum refresh)</t>
+        </is>
+      </c>
+      <c r="H93" s="4" t="inlineStr">
+        <is>
+          <t>404 atau silent ignore, no error popup</t>
+        </is>
+      </c>
+      <c r="I93" s="7" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J93" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K93" s="4" t="inlineStr"/>
+      <c r="L93" s="4" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="inlineStr">
+        <is>
+          <t>ADM-017</t>
+        </is>
+      </c>
+      <c r="B94" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="C94" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D94" s="4" t="inlineStr">
+        <is>
+          <t>CRUD</t>
+        </is>
+      </c>
+      <c r="E94" s="4" t="inlineStr">
+        <is>
+          <t>Create course dengan field kosong (title, description)</t>
+        </is>
+      </c>
+      <c r="F94" s="4" t="inlineStr">
+        <is>
+          <t>Teacher login</t>
+        </is>
+      </c>
+      <c r="G94" s="4" t="inlineStr">
+        <is>
+          <t>1. Buka form Tambah Course
+2. Submit tanpa isi title</t>
+        </is>
+      </c>
+      <c r="H94" s="4" t="inlineStr">
+        <is>
+          <t>Validasi form gagal, error 'Title wajib diisi'</t>
+        </is>
+      </c>
+      <c r="I94" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J94" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K94" s="4" t="inlineStr"/>
+      <c r="L94" s="4" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="inlineStr">
+        <is>
+          <t>ADM-018</t>
+        </is>
+      </c>
+      <c r="B95" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="C95" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D95" s="4" t="inlineStr">
+        <is>
+          <t>Permission</t>
+        </is>
+      </c>
+      <c r="E95" s="4" t="inlineStr">
+        <is>
+          <t>Teacher non-admin akses endpoint admin-only</t>
+        </is>
+      </c>
+      <c r="F95" s="4" t="inlineStr">
+        <is>
+          <t>Login as teacher (non-admin)</t>
+        </is>
+      </c>
+      <c r="G95" s="4" t="inlineStr">
+        <is>
+          <t>1. Kirim POST ke /admin/users (admin only)</t>
+        </is>
+      </c>
+      <c r="H95" s="4" t="inlineStr">
+        <is>
+          <t>403 Forbidden</t>
+        </is>
+      </c>
+      <c r="I95" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J95" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K95" s="4" t="inlineStr"/>
+      <c r="L95" s="4" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="4" t="inlineStr">
+        <is>
+          <t>ADM-019</t>
+        </is>
+      </c>
+      <c r="B96" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="C96" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D96" s="4" t="inlineStr">
+        <is>
+          <t>Exam</t>
+        </is>
+      </c>
+      <c r="E96" s="4" t="inlineStr">
+        <is>
+          <t>Create exam dengan due_date di masa lalu</t>
+        </is>
+      </c>
+      <c r="F96" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G96" s="4" t="inlineStr">
+        <is>
+          <t>1. Form Tambah Exam, isi due_date kemarin</t>
+        </is>
+      </c>
+      <c r="H96" s="4" t="inlineStr">
+        <is>
+          <t>Validasi gagal, error 'Due date harus di masa depan'</t>
+        </is>
+      </c>
+      <c r="I96" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J96" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K96" s="4" t="inlineStr"/>
+      <c r="L96" s="4" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="4" t="inlineStr">
+        <is>
+          <t>ADM-020</t>
+        </is>
+      </c>
+      <c r="B97" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="C97" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D97" s="4" t="inlineStr">
+        <is>
+          <t>Bulk Upload</t>
+        </is>
+      </c>
+      <c r="E97" s="4" t="inlineStr">
+        <is>
+          <t>Bulk upload dengan CSV format salah</t>
+        </is>
+      </c>
+      <c r="F97" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G97" s="4" t="inlineStr">
+        <is>
+          <t>1. Upload CSV dengan kolom missing / typo</t>
+        </is>
+      </c>
+      <c r="H97" s="4" t="inlineStr">
+        <is>
+          <t>Error report: list baris yang gagal + alasan, partial success atau full fail</t>
+        </is>
+      </c>
+      <c r="I97" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J97" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K97" s="4" t="inlineStr"/>
+      <c r="L97" s="4" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="4" t="inlineStr">
+        <is>
+          <t>ADM-021</t>
+        </is>
+      </c>
+      <c r="B98" s="4" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+      <c r="C98" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D98" s="4" t="inlineStr">
+        <is>
+          <t>Cheating</t>
+        </is>
+      </c>
+      <c r="E98" s="4" t="inlineStr">
+        <is>
+          <t>Cheating report untuk exam yang tidak ada</t>
+        </is>
+      </c>
+      <c r="F98" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G98" s="4" t="inlineStr">
+        <is>
+          <t>1. Buka /dashboard-admin/cheating-report?exam_id=99999</t>
+        </is>
+      </c>
+      <c r="H98" s="4" t="inlineStr">
+        <is>
+          <t>Empty state, pesan 'Belum ada data cheating'</t>
+        </is>
+      </c>
+      <c r="I98" s="7" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J98" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K98" s="4" t="inlineStr"/>
+      <c r="L98" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L71"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4748,7 +6232,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L66"/>
+  <dimension ref="A1:L88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8337,6 +9821,1194 @@
       <c r="K66" s="4" t="inlineStr"/>
       <c r="L66" s="4" t="inlineStr"/>
     </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>API-AUTH-009</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>/auth/login-elearning</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>Login dengan email mengandung SQL injection</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t>{"email": "admin@test.com\" OR 1=1--", "password": "x"}</t>
+        </is>
+      </c>
+      <c r="H67" s="4" t="inlineStr">
+        <is>
+          <t>400 Bad Request (input disanitasi) atau 401 Unauthorized, BUKAN 200 dengan data leak</t>
+        </is>
+      </c>
+      <c r="I67" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J67" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K67" s="4" t="inlineStr"/>
+      <c r="L67" s="4" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>API-AUTH-010</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>/auth/login-elearning</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t>Login tanpa body</t>
+        </is>
+      </c>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G68" s="4" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="H68" s="4" t="inlineStr">
+        <is>
+          <t>400 Bad Request, validation error</t>
+        </is>
+      </c>
+      <c r="I68" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J68" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K68" s="4" t="inlineStr"/>
+      <c r="L68" s="4" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>API-AUTH-011</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>/auth/login-elearning</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>Login dengan Content-Type bukan JSON</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>Content-Type: text/plain, body=raw</t>
+        </is>
+      </c>
+      <c r="H69" s="4" t="inlineStr">
+        <is>
+          <t>415 Unsupported Media Type atau 400 Bad Request</t>
+        </is>
+      </c>
+      <c r="I69" s="7" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J69" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K69" s="4" t="inlineStr"/>
+      <c r="L69" s="4" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>API-AUTH-012</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>/auth/refresh</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t>Refresh dengan token invalid</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G70" s="4" t="inlineStr">
+        <is>
+          <t>{"refresh_token": "invalid"}</t>
+        </is>
+      </c>
+      <c r="H70" s="4" t="inlineStr">
+        <is>
+          <t>401 Unauthorized</t>
+        </is>
+      </c>
+      <c r="I70" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J70" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K70" s="4" t="inlineStr"/>
+      <c r="L70" s="4" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>API-AUTH-013</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>/auth/refresh</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t>Refresh dengan refresh_token expired</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G71" s="4" t="inlineStr">
+        <is>
+          <t>{"refresh_token": "&lt;expired&gt;"}</t>
+        </is>
+      </c>
+      <c r="H71" s="4" t="inlineStr">
+        <is>
+          <t>401 Unauthorized, message: "Refresh token expired"</t>
+        </is>
+      </c>
+      <c r="I71" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J71" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K71" s="4" t="inlineStr"/>
+      <c r="L71" s="4" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>API-STU-010</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>/student/enroll</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t>Enroll tanpa auth (token)</t>
+        </is>
+      </c>
+      <c r="F72" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G72" s="4" t="inlineStr">
+        <is>
+          <t>{"course_id": 1}</t>
+        </is>
+      </c>
+      <c r="H72" s="4" t="inlineStr">
+        <is>
+          <t>401 Unauthorized</t>
+        </is>
+      </c>
+      <c r="I72" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J72" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K72" s="4" t="inlineStr"/>
+      <c r="L72" s="4" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>API-STU-011</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>/student/enroll</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>Enroll dengan course_id bukan number</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G73" s="4" t="inlineStr">
+        <is>
+          <t>{"course_id": "abc"}</t>
+        </is>
+      </c>
+      <c r="H73" s="4" t="inlineStr">
+        <is>
+          <t>400 Bad Request, validation error</t>
+        </is>
+      </c>
+      <c r="I73" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J73" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K73" s="4" t="inlineStr"/>
+      <c r="L73" s="4" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>API-STU-012</t>
+        </is>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>/student/courses/abc</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="inlineStr">
+        <is>
+          <t>Get course dengan ID invalid (non-numeric)</t>
+        </is>
+      </c>
+      <c r="F74" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G74" s="4" t="inlineStr">
+        <is>
+          <t>/student/courses/abc</t>
+        </is>
+      </c>
+      <c r="H74" s="4" t="inlineStr">
+        <is>
+          <t>400 Bad Request atau 404 Not Found</t>
+        </is>
+      </c>
+      <c r="I74" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J74" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K74" s="4" t="inlineStr"/>
+      <c r="L74" s="4" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>API-STU-013</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>/student/content/123</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>Get content yang tidak ada</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G75" s="4" t="inlineStr">
+        <is>
+          <t>/student/content/99999</t>
+        </is>
+      </c>
+      <c r="H75" s="4" t="inlineStr">
+        <is>
+          <t>404 Not Found</t>
+        </is>
+      </c>
+      <c r="I75" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J75" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K75" s="4" t="inlineStr"/>
+      <c r="L75" s="4" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t>API-CBT-010</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>/student/exams-attempt/:id/answers</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>Save answer setelah exam disubmit (race condition)</t>
+        </is>
+      </c>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t>Exam sudah disubmit</t>
+        </is>
+      </c>
+      <c r="G76" s="4" t="inlineStr">
+        <is>
+          <t>{"question_id": "q1", "selected_option_id": ["a"]}</t>
+        </is>
+      </c>
+      <c r="H76" s="4" t="inlineStr">
+        <is>
+          <t>409 Conflict, "Cannot modify submitted exam"</t>
+        </is>
+      </c>
+      <c r="I76" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J76" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K76" s="4" t="inlineStr"/>
+      <c r="L76" s="4" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>API-CBT-011</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>/student/exams-attempt/:id/tab-switch</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>Tab switch spam (50x request dalam 1 detik)</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G77" s="4" t="inlineStr">
+        <is>
+          <t>50x POST dalam 1 detik</t>
+        </is>
+      </c>
+      <c r="H77" s="4" t="inlineStr">
+        <is>
+          <t>Rate limit 429 setelah threshold, atau lives langsung 0</t>
+        </is>
+      </c>
+      <c r="I77" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J77" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K77" s="4" t="inlineStr"/>
+      <c r="L77" s="4" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>API-CBT-012</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>/student/exams-attempt/:id/submit</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>Submit attempt orang lain (IDOR attempt)</t>
+        </is>
+      </c>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>Login as student A</t>
+        </is>
+      </c>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
+          <t>Submit attempt_id milik student B</t>
+        </is>
+      </c>
+      <c r="H78" s="4" t="inlineStr">
+        <is>
+          <t>403 Forbidden, "Cannot access other user attempt"</t>
+        </is>
+      </c>
+      <c r="I78" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J78" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K78" s="4" t="inlineStr"/>
+      <c r="L78" s="4" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>API-CBT-013</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>/student/exams-attempt/:id/answers</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>Save answer untuk question yang tidak ada di exam</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>{"question_id": "fake_id_999", "selected_option_id": ["a"]}</t>
+        </is>
+      </c>
+      <c r="H79" s="4" t="inlineStr">
+        <is>
+          <t>400 Bad Request, "Invalid question"</t>
+        </is>
+      </c>
+      <c r="I79" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J79" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K79" s="4" t="inlineStr"/>
+      <c r="L79" s="4" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>API-CBT-014</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>/student/exams-attempt/:id/answers</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>Save answer dengan selected_option_id kosong</t>
+        </is>
+      </c>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G80" s="4" t="inlineStr">
+        <is>
+          <t>{"question_id": "q1", "selected_option_id": []}</t>
+        </is>
+      </c>
+      <c r="H80" s="4" t="inlineStr">
+        <is>
+          <t>400 Bad Request, validation error</t>
+        </is>
+      </c>
+      <c r="I80" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J80" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K80" s="4" t="inlineStr"/>
+      <c r="L80" s="4" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>API-CBT-015</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>/upcoming-exam</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>Get upcoming exam tanpa auth</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G81" s="4" t="inlineStr">
+        <is>
+          <t>(no token)</t>
+        </is>
+      </c>
+      <c r="H81" s="4" t="inlineStr">
+        <is>
+          <t>401 Unauthorized</t>
+        </is>
+      </c>
+      <c r="I81" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J81" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K81" s="4" t="inlineStr"/>
+      <c r="L81" s="4" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t>API-TCH-009</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>/teacher/add-course</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="inlineStr">
+        <is>
+          <t>Create course dengan title kosong</t>
+        </is>
+      </c>
+      <c r="F82" s="4" t="inlineStr">
+        <is>
+          <t>Teacher login</t>
+        </is>
+      </c>
+      <c r="G82" s="4" t="inlineStr">
+        <is>
+          <t>{"title": "", "description": "...", "subject": "math"}</t>
+        </is>
+      </c>
+      <c r="H82" s="4" t="inlineStr">
+        <is>
+          <t>400 Bad Request, "Title required"</t>
+        </is>
+      </c>
+      <c r="I82" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J82" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K82" s="4" t="inlineStr"/>
+      <c r="L82" s="4" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>API-TCH-010</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>/teacher/courses/9999</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>Update course yang tidak ada</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G83" s="4" t="inlineStr">
+        <is>
+          <t>{"title": "Updated"}</t>
+        </is>
+      </c>
+      <c r="H83" s="4" t="inlineStr">
+        <is>
+          <t>404 Not Found</t>
+        </is>
+      </c>
+      <c r="I83" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J83" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K83" s="4" t="inlineStr"/>
+      <c r="L83" s="4" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>API-TCH-011</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>/teacher/courses/:id</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="inlineStr">
+        <is>
+          <t>Delete course yang punya student enrolled</t>
+        </is>
+      </c>
+      <c r="F84" s="4" t="inlineStr">
+        <is>
+          <t>Course ada student</t>
+        </is>
+      </c>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
+          <t>(no body)</t>
+        </is>
+      </c>
+      <c r="H84" s="4" t="inlineStr">
+        <is>
+          <t>409 Conflict, "Cannot delete course with active students" (atau soft delete + warning)</t>
+        </is>
+      </c>
+      <c r="I84" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J84" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K84" s="4" t="inlineStr"/>
+      <c r="L84" s="4" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>API-TCH-012</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>/teacher/add-course</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="inlineStr">
+        <is>
+          <t>Create course tanpa auth</t>
+        </is>
+      </c>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>{"title": "..."}</t>
+        </is>
+      </c>
+      <c r="H85" s="4" t="inlineStr">
+        <is>
+          <t>401 Unauthorized</t>
+        </is>
+      </c>
+      <c r="I85" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J85" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K85" s="4" t="inlineStr"/>
+      <c r="L85" s="4" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="inlineStr">
+        <is>
+          <t>API-EXM-011</t>
+        </is>
+      </c>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>/teacher/courses/:id/exam</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E86" s="4" t="inlineStr">
+        <is>
+          <t>Create exam dengan duration &lt;= 0</t>
+        </is>
+      </c>
+      <c r="F86" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G86" s="4" t="inlineStr">
+        <is>
+          <t>{"title": "UTS", "duration": 0, "due_date": "2026-12-31"}</t>
+        </is>
+      </c>
+      <c r="H86" s="4" t="inlineStr">
+        <is>
+          <t>400 Bad Request, "Duration must be &gt; 0"</t>
+        </is>
+      </c>
+      <c r="I86" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J86" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K86" s="4" t="inlineStr"/>
+      <c r="L86" s="4" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>API-EXM-012</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>/teacher/courses/:id/exam</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E87" s="4" t="inlineStr">
+        <is>
+          <t>Create exam dengan due_date di masa lalu</t>
+        </is>
+      </c>
+      <c r="F87" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G87" s="4" t="inlineStr">
+        <is>
+          <t>{"title": "UTS", "duration": 60, "due_date": "2020-01-01"}</t>
+        </is>
+      </c>
+      <c r="H87" s="4" t="inlineStr">
+        <is>
+          <t>400 Bad Request, "Due date must be in future"</t>
+        </is>
+      </c>
+      <c r="I87" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J87" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K87" s="4" t="inlineStr"/>
+      <c r="L87" s="4" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="inlineStr">
+        <is>
+          <t>API-EXM-013</t>
+        </is>
+      </c>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>/teacher/exams/:id/questions</t>
+        </is>
+      </c>
+      <c r="C88" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E88" s="4" t="inlineStr">
+        <is>
+          <t>Add question tanpa options untuk single_choice</t>
+        </is>
+      </c>
+      <c r="F88" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G88" s="4" t="inlineStr">
+        <is>
+          <t>{"question_text": "Test", "question_type": "single", "options": []}</t>
+        </is>
+      </c>
+      <c r="H88" s="4" t="inlineStr">
+        <is>
+          <t>400 Bad Request, "Options required for single choice"</t>
+        </is>
+      </c>
+      <c r="I88" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J88" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K88" s="4" t="inlineStr"/>
+      <c r="L88" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L66"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add 15 API test cases to Arteri (10 security negative + 5 edge)
</commit_message>
<xml_diff>
--- a/projects/arteri-elearning/test-cases.xlsx
+++ b/projects/arteri-elearning/test-cases.xlsx
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>87</v>
+        <v>102</v>
       </c>
     </row>
     <row r="14">
@@ -628,7 +628,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>135</v>
+        <v>199</v>
       </c>
     </row>
     <row r="15"/>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="30">
@@ -767,7 +767,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="31">
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
     </row>
     <row r="33">
@@ -797,7 +797,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="34">
@@ -817,9 +817,13 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1</v>
-      </c>
-    </row>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6232,7 +6236,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L88"/>
+  <dimension ref="A1:L103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11009,6 +11013,816 @@
       <c r="K88" s="4" t="inlineStr"/>
       <c r="L88" s="4" t="inlineStr"/>
     </row>
+    <row r="89">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>API-AUTH-014</t>
+        </is>
+      </c>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>/auth/me</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E89" s="4" t="inlineStr">
+        <is>
+          <t>JWT replay attack (reuse token setelah logout)</t>
+        </is>
+      </c>
+      <c r="F89" s="4" t="inlineStr">
+        <is>
+          <t>User logout, simpan token lama</t>
+        </is>
+      </c>
+      <c r="G89" s="4" t="inlineStr">
+        <is>
+          <t>(with logged-out token)</t>
+        </is>
+      </c>
+      <c r="H89" s="4" t="inlineStr">
+        <is>
+          <t>401 Unauthorized, message: "Token revoked" (server harus track revoked tokens)</t>
+        </is>
+      </c>
+      <c r="I89" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J89" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K89" s="4" t="inlineStr"/>
+      <c r="L89" s="4" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="inlineStr">
+        <is>
+          <t>API-AUTH-015</t>
+        </is>
+      </c>
+      <c r="B90" s="4" t="inlineStr">
+        <is>
+          <t>/auth/register</t>
+        </is>
+      </c>
+      <c r="C90" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E90" s="4" t="inlineStr">
+        <is>
+          <t>Mass assignment attack (kirim field role=admin)</t>
+        </is>
+      </c>
+      <c r="F90" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G90" s="4" t="inlineStr">
+        <is>
+          <t>{"name": "x", "email": "x@test.com", "password": "Valid123!", "role": "admin", "is_admin": true}</t>
+        </is>
+      </c>
+      <c r="H90" s="4" t="inlineStr">
+        <is>
+          <t>201 Created, TAPI role yang tersimpan = "student" (default), field tambahan diabaikan/di-strip</t>
+        </is>
+      </c>
+      <c r="I90" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J90" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K90" s="4" t="inlineStr"/>
+      <c r="L90" s="4" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <t>API-STU-014</t>
+        </is>
+      </c>
+      <c r="B91" s="4" t="inlineStr">
+        <is>
+          <t>/courses/browse</t>
+        </is>
+      </c>
+      <c r="C91" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E91" s="4" t="inlineStr">
+        <is>
+          <t>SQL injection di search query</t>
+        </is>
+      </c>
+      <c r="F91" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G91" s="4" t="inlineStr">
+        <is>
+          <t>?search=test%27%20OR%20%271%27%3D%271</t>
+        </is>
+      </c>
+      <c r="H91" s="4" t="inlineStr">
+        <is>
+          <t>200 OK dengan list kosong atau error, TIDAK return semua data (sanitized)</t>
+        </is>
+      </c>
+      <c r="I91" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J91" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K91" s="4" t="inlineStr"/>
+      <c r="L91" s="4" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="inlineStr">
+        <is>
+          <t>API-STU-015</t>
+        </is>
+      </c>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t>/courses/browse</t>
+        </is>
+      </c>
+      <c r="C92" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E92" s="4" t="inlineStr">
+        <is>
+          <t>SQL injection dengan UNION SELECT</t>
+        </is>
+      </c>
+      <c r="F92" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G92" s="4" t="inlineStr">
+        <is>
+          <t>?search=test%27%20UNION%20SELECT%20*%20FROM%20users--</t>
+        </is>
+      </c>
+      <c r="H92" s="4" t="inlineStr">
+        <is>
+          <t>400 Bad Request atau 200 dengan list kosong, BUKAN data user terexpose</t>
+        </is>
+      </c>
+      <c r="I92" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J92" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K92" s="4" t="inlineStr"/>
+      <c r="L92" s="4" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr">
+        <is>
+          <t>API-CBT-016</t>
+        </is>
+      </c>
+      <c r="B93" s="4" t="inlineStr">
+        <is>
+          <t>/upcoming-exam</t>
+        </is>
+      </c>
+      <c r="C93" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E93" s="4" t="inlineStr">
+        <is>
+          <t>CORS bypass attempt (Origin: attacker.com)</t>
+        </is>
+      </c>
+      <c r="F93" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G93" s="4" t="inlineStr">
+        <is>
+          <t>Header Origin: https://attacker.com</t>
+        </is>
+      </c>
+      <c r="H93" s="4" t="inlineStr">
+        <is>
+          <t>Response TIDAK punya Access-Control-Allow-Origin: https://attacker.com (CORS strict)</t>
+        </is>
+      </c>
+      <c r="I93" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J93" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K93" s="4" t="inlineStr"/>
+      <c r="L93" s="4" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="inlineStr">
+        <is>
+          <t>API-CBT-017</t>
+        </is>
+      </c>
+      <c r="B94" s="4" t="inlineStr">
+        <is>
+          <t>/student/exams-attempt/:id/answers</t>
+        </is>
+      </c>
+      <c r="C94" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D94" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E94" s="4" t="inlineStr">
+        <is>
+          <t>Negative index di question (manipulate question_id)</t>
+        </is>
+      </c>
+      <c r="F94" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G94" s="4" t="inlineStr">
+        <is>
+          <t>{"question_id": -1, "selected_option_id": ["a"]}</t>
+        </is>
+      </c>
+      <c r="H94" s="4" t="inlineStr">
+        <is>
+          <t>400 Bad Request, "Invalid question_id"</t>
+        </is>
+      </c>
+      <c r="I94" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J94" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K94" s="4" t="inlineStr"/>
+      <c r="L94" s="4" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="inlineStr">
+        <is>
+          <t>API-CBT-018</t>
+        </is>
+      </c>
+      <c r="B95" s="4" t="inlineStr">
+        <is>
+          <t>/student/exams-attempt/:id/answers</t>
+        </is>
+      </c>
+      <c r="C95" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D95" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E95" s="4" t="inlineStr">
+        <is>
+          <t>Mass assignment (kirim is_correct, score field)</t>
+        </is>
+      </c>
+      <c r="F95" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G95" s="4" t="inlineStr">
+        <is>
+          <t>{"question_id": "q1", "selected_option_id": ["a"], "is_correct": true, "score": 100}</t>
+        </is>
+      </c>
+      <c r="H95" s="4" t="inlineStr">
+        <is>
+          <t>201 Created (atau 200), TAPI score dan is_correct di-strip (server-side compute)</t>
+        </is>
+      </c>
+      <c r="I95" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J95" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K95" s="4" t="inlineStr"/>
+      <c r="L95" s="4" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="4" t="inlineStr">
+        <is>
+          <t>API-TCH-013</t>
+        </is>
+      </c>
+      <c r="B96" s="4" t="inlineStr">
+        <is>
+          <t>/admin/users</t>
+        </is>
+      </c>
+      <c r="C96" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D96" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E96" s="4" t="inlineStr">
+        <is>
+          <t>Privilege escalation (teacher non-admin coba akses admin endpoint)</t>
+        </is>
+      </c>
+      <c r="F96" s="4" t="inlineStr">
+        <is>
+          <t>Login as teacher biasa (non-admin)</t>
+        </is>
+      </c>
+      <c r="G96" s="4" t="inlineStr">
+        <is>
+          <t>(with teacher token)</t>
+        </is>
+      </c>
+      <c r="H96" s="4" t="inlineStr">
+        <is>
+          <t>403 Forbidden, "Admin access required"</t>
+        </is>
+      </c>
+      <c r="I96" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J96" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K96" s="4" t="inlineStr"/>
+      <c r="L96" s="4" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="4" t="inlineStr">
+        <is>
+          <t>API-TCH-014</t>
+        </is>
+      </c>
+      <c r="B97" s="4" t="inlineStr">
+        <is>
+          <t>/auth/login-elearning</t>
+        </is>
+      </c>
+      <c r="C97" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D97" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E97" s="4" t="inlineStr">
+        <is>
+          <t>Timing attack (response time beda untuk valid vs invalid user)</t>
+        </is>
+      </c>
+      <c r="F97" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G97" s="4" t="inlineStr">
+        <is>
+          <t>Compare timing: email valid + random password vs random email</t>
+        </is>
+      </c>
+      <c r="H97" s="4" t="inlineStr">
+        <is>
+          <t>Response time konsisten (&lt; 100ms difference) untuk valid dan invalid user (timing-safe comparison)</t>
+        </is>
+      </c>
+      <c r="I97" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J97" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K97" s="4" t="inlineStr"/>
+      <c r="L97" s="4" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="4" t="inlineStr">
+        <is>
+          <t>API-EXM-014</t>
+        </is>
+      </c>
+      <c r="B98" s="4" t="inlineStr">
+        <is>
+          <t>/teacher/courses/:id/exam</t>
+        </is>
+      </c>
+      <c r="C98" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D98" s="4" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="E98" s="4" t="inlineStr">
+        <is>
+          <t>Mass assignment (kirim is_published=true di body create)</t>
+        </is>
+      </c>
+      <c r="F98" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G98" s="4" t="inlineStr">
+        <is>
+          <t>{"title": "x", "duration": 60, "due_date": "2026-12-31", "is_published": true, "created_by": "fake_id"}</t>
+        </is>
+      </c>
+      <c r="H98" s="4" t="inlineStr">
+        <is>
+          <t>201 Created, TAPI is_published default false (draft), created_by di-strip (server ambil dari token)</t>
+        </is>
+      </c>
+      <c r="I98" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="J98" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K98" s="4" t="inlineStr"/>
+      <c r="L98" s="4" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t>API-AUTH-016</t>
+        </is>
+      </c>
+      <c r="B99" s="4" t="inlineStr">
+        <is>
+          <t>/auth/login-elearning</t>
+        </is>
+      </c>
+      <c r="C99" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D99" s="4" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="E99" s="4" t="inlineStr">
+        <is>
+          <t>Empty body (no Content-Length, no body)</t>
+        </is>
+      </c>
+      <c r="F99" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G99" s="4" t="inlineStr">
+        <is>
+          <t>(empty body, no Content-Type)</t>
+        </is>
+      </c>
+      <c r="H99" s="4" t="inlineStr">
+        <is>
+          <t>400 Bad Request atau 411 Length Required, TIDAK crash server</t>
+        </is>
+      </c>
+      <c r="I99" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J99" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K99" s="4" t="inlineStr"/>
+      <c r="L99" s="4" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="4" t="inlineStr">
+        <is>
+          <t>API-STU-016</t>
+        </is>
+      </c>
+      <c r="B100" s="4" t="inlineStr">
+        <is>
+          <t>/courses/browse</t>
+        </is>
+      </c>
+      <c r="C100" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D100" s="4" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="E100" s="4" t="inlineStr">
+        <is>
+          <t>Max size query string (&gt; 8KB)</t>
+        </is>
+      </c>
+      <c r="F100" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G100" s="4" t="inlineStr">
+        <is>
+          <t>?search=&lt;8000 character random string&gt;</t>
+        </is>
+      </c>
+      <c r="H100" s="4" t="inlineStr">
+        <is>
+          <t>200 OK dengan list kosong (atau 414 URI Too Long), server tidak crash</t>
+        </is>
+      </c>
+      <c r="I100" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J100" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K100" s="4" t="inlineStr"/>
+      <c r="L100" s="4" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="4" t="inlineStr">
+        <is>
+          <t>API-STU-017</t>
+        </is>
+      </c>
+      <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>/student/notes</t>
+        </is>
+      </c>
+      <c r="C101" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D101" s="4" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="E101" s="4" t="inlineStr">
+        <is>
+          <t>Unicode/emoji di input</t>
+        </is>
+      </c>
+      <c r="F101" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G101" s="4" t="inlineStr">
+        <is>
+          <t>{"topic_id": 1, "content": "测试 🎓 العربية 한국어 🦄"}</t>
+        </is>
+      </c>
+      <c r="H101" s="4" t="inlineStr">
+        <is>
+          <t>201 Created, content tersimpan dengan benar (UTF-8 support verified)</t>
+        </is>
+      </c>
+      <c r="I101" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J101" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K101" s="4" t="inlineStr"/>
+      <c r="L101" s="4" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="4" t="inlineStr">
+        <is>
+          <t>API-CBT-019</t>
+        </is>
+      </c>
+      <c r="B102" s="4" t="inlineStr">
+        <is>
+          <t>/teacher/exams/:id/questions</t>
+        </is>
+      </c>
+      <c r="C102" s="4" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D102" s="4" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="E102" s="4" t="inlineStr">
+        <is>
+          <t>Very long question text (10,000 karakter)</t>
+        </is>
+      </c>
+      <c r="F102" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G102" s="4" t="inlineStr">
+        <is>
+          <t>{"question_text": "&lt;10K random chars&gt;", "question_type": "single", "options": [...], "correct": "a"}</t>
+        </is>
+      </c>
+      <c r="H102" s="4" t="inlineStr">
+        <is>
+          <t>201 Created atau 413 Payload Too Large (kalau ada max length, return 400 dengan pesan jelas)</t>
+        </is>
+      </c>
+      <c r="I102" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J102" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K102" s="4" t="inlineStr"/>
+      <c r="L102" s="4" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="4" t="inlineStr">
+        <is>
+          <t>API-TCH-015</t>
+        </is>
+      </c>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>/student/courses/99999999999999999999</t>
+        </is>
+      </c>
+      <c r="C103" s="4" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="D103" s="4" t="inlineStr">
+        <is>
+          <t>Edge</t>
+        </is>
+      </c>
+      <c r="E103" s="4" t="inlineStr">
+        <is>
+          <t>Integer overflow pada path parameter</t>
+        </is>
+      </c>
+      <c r="F103" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G103" s="4" t="inlineStr">
+        <is>
+          <t>/student/courses/99999999999999999999</t>
+        </is>
+      </c>
+      <c r="H103" s="4" t="inlineStr">
+        <is>
+          <t>400 Bad Request (invalid ID) atau 404 Not Found, TIDAK crash dengan NumberFormatError</t>
+        </is>
+      </c>
+      <c r="I103" s="6" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="J103" s="4" t="inlineStr">
+        <is>
+          <t>Belum Dieksekusi</t>
+        </is>
+      </c>
+      <c r="K103" s="4" t="inlineStr"/>
+      <c r="L103" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L66"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>